<commit_message>
Added config reader and validation for data from excel sheet
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/StockData.xlsx
+++ b/src/test/resources/testdata/StockData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\final-capstone-project\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87031F62-0029-4573-A172-2C88C8E9CF83}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3387992-D7C9-4591-B0BC-5420F5BAAC8B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4470" xr2:uid="{F069813A-FF43-40E1-8DE5-2B77017C3FB6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Reliance</t>
   </si>
@@ -34,6 +34,15 @@
   </si>
   <si>
     <t>StockName</t>
+  </si>
+  <si>
+    <t>ExpectedHigh</t>
+  </si>
+  <si>
+    <t>ExpectedLow</t>
+  </si>
+  <si>
+    <t>Tata Motors</t>
   </si>
 </sst>
 </file>
@@ -69,8 +78,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,22 +395,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F29E7EC-0113-4FE7-BDD6-F41906930C01}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="1">
+        <v>2006.45</v>
+      </c>
+      <c r="C2">
+        <v>1307</v>
+      </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1551</v>
+      </c>
+      <c r="C3">
+        <v>1114.8499999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>774.45</v>
+      </c>
+      <c r="C4">
+        <v>702.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>